<commit_message>
Fix multi-battle warnings and Safari rotations v0.8.7
</commit_message>
<xml_diff>
--- a/tools/MUSH_WARtool_Google_Sheet_Template.xlsx
+++ b/tools/MUSH_WARtool_Google_Sheet_Template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Re359547c473e490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH To My Surprise" sheetId="2" r:id="R11387c7b145540fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH More Like It" sheetId="3" r:id="Rd41a32002be144ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" r:id="R18bcd451b1424a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosters" sheetId="5" r:id="Rcb0d4a78d91e494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokémon" sheetId="6" r:id="Ra337f4ca3e3140af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Rdd660e9009754feb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH To My Surprise" sheetId="2" r:id="R11446845e2bf4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH More Like It" sheetId="3" r:id="R08de7cf3874845d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" r:id="Raf8291d36aae4f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosters" sheetId="5" r:id="R235aaba932f24f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokémon" sheetId="6" r:id="Re18ae3dbaf9c4312"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,67 +104,27 @@
   <x:borders count="18">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="139">
+  <x:cellXfs count="140">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -512,6 +472,13 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -519,14 +486,14 @@
   <x:dxfs count="2">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F6F0"/>
         </x:patternFill>
       </x:fill>
@@ -11342,7 +11309,7 @@
   <x:cols>
     <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="56" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -11609,10 +11576,32 @@
         <x:v>Fossil revivals/hour; editable</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="36" t="str">
+        <x:v>johtoSafariRotationalTier</x:v>
+      </x:c>
+      <x:c r="B25" s="36" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C25" s="36" t="str">
+        <x:v>Tier estimate for the undocumented Johto Safari 10% slot; -1 leaves it unscored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="36" t="str">
+        <x:v>greatMarshRotationalTier</x:v>
+      </x:c>
+      <x:c r="B26" s="36" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C26" s="36" t="str">
+        <x:v>Tier estimate for the undocumented Great Marsh 20% slot; -1 leaves it unscored</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf60fc595d46340f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R963d330590d146cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22322,7 +22311,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d384874a5404184"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R269805b6a81d40ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use species-specific Safari catch rates v0.8.8
</commit_message>
<xml_diff>
--- a/tools/MUSH_WARtool_Google_Sheet_Template.xlsx
+++ b/tools/MUSH_WARtool_Google_Sheet_Template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Rdd660e9009754feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH To My Surprise" sheetId="2" r:id="R11446845e2bf4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH More Like It" sheetId="3" r:id="R08de7cf3874845d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" r:id="Raf8291d36aae4f26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosters" sheetId="5" r:id="R235aaba932f24f13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokémon" sheetId="6" r:id="Re18ae3dbaf9c4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R0d4fb2b71dd140d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH To My Surprise" sheetId="2" r:id="R7bb0b057a8834491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MÜSH More Like It" sheetId="3" r:id="R35010e72a3f44e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" r:id="R47754f12a05c4d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosters" sheetId="5" r:id="Rc35d8ea9220a49e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokémon" sheetId="6" r:id="R6d4964bd8b004a86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -124,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="140">
+  <x:cellXfs count="143">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -479,6 +479,15 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11313,295 +11322,317 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="97" t="str">
+      <x:c r="A1" s="140" t="str">
         <x:v>Setting</x:v>
       </x:c>
-      <x:c r="B1" s="98" t="str">
+      <x:c r="B1" s="140" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="C1" s="99" t="str">
+      <x:c r="C1" s="140" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="51" t="str">
+      <x:c r="A2" s="36" t="str">
         <x:v>baseShinyDenominator</x:v>
       </x:c>
-      <x:c r="B2" s="52" t="n">
+      <x:c r="B2" s="36" t="n">
         <x:v>30000</x:v>
       </x:c>
-      <x:c r="C2" s="53" t="str">
+      <x:c r="C2" s="36" t="str">
         <x:v>Official base shiny denominator</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="51" t="str">
+      <x:c r="A3" s="36" t="str">
         <x:v>eventWildBoost</x:v>
       </x:c>
-      <x:c r="B3" s="117" t="n">
+      <x:c r="B3" s="141" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="C3" s="53" t="str">
+      <x:c r="C3" s="36" t="str">
         <x:v>Wild-only Shiny Wars boost; Fossil ignores this</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="51" t="str">
+      <x:c r="A4" s="36" t="str">
         <x:v>uniqueBonus</x:v>
       </x:c>
-      <x:c r="B4" s="52" t="n">
+      <x:c r="B4" s="36" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C4" s="53" t="str">
+      <x:c r="C4" s="36" t="str">
         <x:v>First evolution line caught by that competition team</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="51" t="str">
+      <x:c r="A5" s="36" t="str">
         <x:v>secretBonus</x:v>
       </x:c>
-      <x:c r="B5" s="52" t="n">
+      <x:c r="B5" s="36" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="36" t="str">
         <x:v>Secret Shiny bonus</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="51" t="str">
+      <x:c r="A6" s="36" t="str">
         <x:v>secretChance</x:v>
       </x:c>
-      <x:c r="B6" s="119" t="n">
+      <x:c r="B6" s="142" t="n">
         <x:v>0.0625</x:v>
       </x:c>
-      <x:c r="C6" s="53" t="str">
+      <x:c r="C6" s="36" t="str">
         <x:v>Expected-value assumption: 1/16</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="51" t="str">
+      <x:c r="A7" s="36" t="str">
         <x:v>safariBonus</x:v>
       </x:c>
-      <x:c r="B7" s="52" t="n">
+      <x:c r="B7" s="36" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C7" s="53" t="str">
+      <x:c r="C7" s="36" t="str">
         <x:v>Successful Safari shiny catch bonus</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="51" t="str">
+      <x:c r="A8" s="36" t="str">
+        <x:v>safariCatchModel</x:v>
+      </x:c>
+      <x:c r="B8" s="141" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="36" t="str">
+        <x:v>1 = matched species estimates plus fallback; 0 = one global catch override</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="36" t="str">
+        <x:v>safariUnknownCatchChance</x:v>
+      </x:c>
+      <x:c r="B9" s="36" t="n">
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="C9" s="36" t="str">
+        <x:v>Fallback success chance for unknown rotationals, unmatched species, Kanto and Hoenn Safari</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="36" t="str">
         <x:v>safariCatchChance</x:v>
       </x:c>
-      <x:c r="B8" s="117" t="n">
+      <x:c r="B10" s="36" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="53" t="str">
-        <x:v>Editable global Safari success assumption</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="51" t="str">
+      <x:c r="C10" s="36" t="str">
+        <x:v>Global success override; used only when safariCatchModel is 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="36" t="str">
+        <x:v>johtoSafariRotationalTier</x:v>
+      </x:c>
+      <x:c r="B11" s="36" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C11" s="36" t="str">
+        <x:v>Tier estimate for the undocumented Johto Safari 10% slot; -1 leaves it unscored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="36" t="str">
+        <x:v>greatMarshRotationalTier</x:v>
+      </x:c>
+      <x:c r="B12" s="36" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C12" s="36" t="str">
+        <x:v>Tier estimate for the undocumented Great Marsh 20% slot; -1 leaves it unscored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="36" t="str">
         <x:v>method.5x Horde</x:v>
       </x:c>
-      <x:c r="B9" s="52" t="n">
+      <x:c r="B13" s="36" t="n">
         <x:v>1200</x:v>
       </x:c>
-      <x:c r="C9" s="53" t="str">
+      <x:c r="C13" s="36" t="str">
         <x:v>Standard optimized 5× Horde speed</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="51" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="36" t="str">
         <x:v>method.5x Horde (Slowed)</x:v>
       </x:c>
-      <x:c r="B10" s="52" t="n">
+      <x:c r="B14" s="36" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="C10" s="53" t="str">
+      <x:c r="C14" s="36" t="str">
         <x:v>Slower 5× Horde spot/setup</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="51" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="36" t="str">
         <x:v>method.3x Horde</x:v>
       </x:c>
-      <x:c r="B11" s="52" t="n">
+      <x:c r="B15" s="36" t="n">
         <x:v>720</x:v>
       </x:c>
-      <x:c r="C11" s="53" t="str">
+      <x:c r="C15" s="36" t="str">
         <x:v>Standard optimized 3× Horde speed</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="51" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="36" t="str">
         <x:v>method.3x Horde (Slowed)</x:v>
       </x:c>
-      <x:c r="B12" s="52" t="n">
+      <x:c r="B16" s="36" t="n">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="C12" s="53" t="str">
+      <x:c r="C16" s="36" t="str">
         <x:v>Slower 3× Horde spot/setup</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="51" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="36" t="str">
         <x:v>method.Lure Singles</x:v>
       </x:c>
-      <x:c r="B13" s="52" t="n">
+      <x:c r="B17" s="36" t="n">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="C13" s="53" t="str">
+      <x:c r="C17" s="36" t="str">
         <x:v>Walking/surfing Lure singles</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="51" t="str">
+    <x:row r="18">
+      <x:c r="A18" s="36" t="str">
         <x:v>method.Singles</x:v>
       </x:c>
-      <x:c r="B14" s="52" t="n">
+      <x:c r="B18" s="36" t="n">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="C14" s="53" t="str">
+      <x:c r="C18" s="36" t="str">
         <x:v>Ordinary single encounters</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="51" t="str">
+    <x:row r="19">
+      <x:c r="A19" s="36" t="str">
         <x:v>method.Safari Singles</x:v>
       </x:c>
-      <x:c r="B15" s="52" t="n">
+      <x:c r="B19" s="36" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="C15" s="53" t="str">
+      <x:c r="C19" s="36" t="str">
         <x:v>Ordinary Safari singles</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="51" t="str">
+    <x:row r="20">
+      <x:c r="A20" s="36" t="str">
         <x:v>method.Lure Safari Singles</x:v>
       </x:c>
-      <x:c r="B16" s="52" t="n">
+      <x:c r="B20" s="36" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="C16" s="53" t="str">
+      <x:c r="C20" s="36" t="str">
         <x:v>Safari with Lure</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="51" t="str">
+    <x:row r="21">
+      <x:c r="A21" s="36" t="str">
         <x:v>method.Fishing</x:v>
       </x:c>
-      <x:c r="B17" s="52" t="n">
+      <x:c r="B21" s="36" t="n">
         <x:v>270</x:v>
       </x:c>
-      <x:c r="C17" s="53" t="str">
+      <x:c r="C21" s="36" t="str">
         <x:v>Fishing without Lure or Chum</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="51" t="str">
+    <x:row r="22">
+      <x:c r="A22" s="36" t="str">
         <x:v>method.Fishing + Lure</x:v>
       </x:c>
-      <x:c r="B18" s="52" t="n">
+      <x:c r="B22" s="36" t="n">
         <x:v>340</x:v>
       </x:c>
-      <x:c r="C18" s="53" t="str">
+      <x:c r="C22" s="36" t="str">
         <x:v>Editable starting assumption</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="51" t="str">
+    <x:row r="23">
+      <x:c r="A23" s="36" t="str">
         <x:v>method.Fishing + Chum Bucket</x:v>
       </x:c>
-      <x:c r="B19" s="52" t="n">
+      <x:c r="B23" s="36" t="n">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="C19" s="53" t="str">
+      <x:c r="C23" s="36" t="str">
         <x:v>Editable starting assumption</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="51" t="str">
+    <x:row r="24">
+      <x:c r="A24" s="36" t="str">
         <x:v>method.Fishing + Lure + Chum Bucket</x:v>
       </x:c>
-      <x:c r="B20" s="52" t="n">
+      <x:c r="B24" s="36" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="C20" s="53" t="str">
+      <x:c r="C24" s="36" t="str">
         <x:v>Editable starting assumption</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="51" t="str">
-        <x:v>method.Rock Smash</x:v>
-      </x:c>
-      <x:c r="B21" s="52" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="C21" s="53" t="str">
-        <x:v>Editable starting assumption</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="51" t="str">
-        <x:v>method.Headbutt</x:v>
-      </x:c>
-      <x:c r="B22" s="52" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="C22" s="53" t="str">
-        <x:v>Editable starting assumption</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="51" t="str">
-        <x:v>method.Honey Tree</x:v>
-      </x:c>
-      <x:c r="B23" s="52" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="C23" s="53" t="str">
-        <x:v>Active encounter assumption; waiting time excluded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="121" t="str">
-        <x:v>method.Fossil</x:v>
-      </x:c>
-      <x:c r="B24" s="102" t="n">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="C24" s="103" t="str">
-        <x:v>Fossil revivals/hour; editable</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="36" t="str">
-        <x:v>johtoSafariRotationalTier</x:v>
+        <x:v>method.Rock Smash</x:v>
       </x:c>
       <x:c r="B25" s="36" t="n">
-        <x:v>-1</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C25" s="36" t="str">
-        <x:v>Tier estimate for the undocumented Johto Safari 10% slot; -1 leaves it unscored</x:v>
+        <x:v>Editable starting assumption</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="36" t="str">
-        <x:v>greatMarshRotationalTier</x:v>
+        <x:v>method.Headbutt</x:v>
       </x:c>
       <x:c r="B26" s="36" t="n">
-        <x:v>-1</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C26" s="36" t="str">
-        <x:v>Tier estimate for the undocumented Great Marsh 20% slot; -1 leaves it unscored</x:v>
+        <x:v>Editable starting assumption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="36" t="str">
+        <x:v>method.Honey Tree</x:v>
+      </x:c>
+      <x:c r="B27" s="36" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C27" s="36" t="str">
+        <x:v>Active encounter assumption; waiting time excluded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="36" t="str">
+        <x:v>method.Fossil</x:v>
+      </x:c>
+      <x:c r="B28" s="36" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C28" s="36" t="str">
+        <x:v>Fossil revivals/hour; editable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R963d330590d146cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6312322498c4105"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22311,7 +22342,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R269805b6a81d40ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d611245a0d4e70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>